<commit_message>
Criamos o código para subir aba gastos da tabela do cliente
</commit_message>
<xml_diff>
--- a/01_clientes/01_restaurante_teste_ativo/Planilha_Operacional_Restaurante_Teste.xlsx
+++ b/01_clientes/01_restaurante_teste_ativo/Planilha_Operacional_Restaurante_Teste.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucoes" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="158">
   <si>
     <t>PASSO</t>
   </si>
@@ -1220,7 +1220,8 @@
   <dimension ref="A1:I411"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="12" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="3" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.44140625" customWidth="1"/>
     <col min="5" max="5" width="13.21875" bestFit="1" customWidth="1"/>
@@ -1505,7 +1506,9 @@
       <c r="C11" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="D11" s="7"/>
+      <c r="D11" s="7" t="s">
+        <v>156</v>
+      </c>
       <c r="E11" s="7">
         <v>3</v>
       </c>
@@ -1555,7 +1558,9 @@
       <c r="C13" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="D13" s="7"/>
+      <c r="D13" s="7" t="s">
+        <v>156</v>
+      </c>
       <c r="E13" s="7">
         <v>4</v>
       </c>
@@ -3559,8 +3564,9 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.88671875" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="4" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.109375" customWidth="1"/>
+    <col min="3" max="3" width="27.88671875" customWidth="1"/>
+    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="12" customWidth="1"/>
   </cols>

</xml_diff>